<commit_message>
Update Banking Stress Testing modal with charts and Excel dashboard
</commit_message>
<xml_diff>
--- a/Banking_Stress_Testing_2024.xlsx
+++ b/Banking_Stress_Testing_2024.xlsx
@@ -16,27 +16,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
-  <si>
-    <t>0.0%</t>
-  </si>
-  <si>
-    <t>0.5%</t>
-  </si>
-  <si>
-    <t>1.0%</t>
-  </si>
-  <si>
-    <t>1.5%</t>
-  </si>
-  <si>
-    <t>2.0%</t>
-  </si>
-  <si>
-    <t>2.5%</t>
-  </si>
-  <si>
-    <t>3.0%</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
+  <si>
+    <t>-2.0%</t>
+  </si>
+  <si>
+    <t>-1.5%</t>
+  </si>
+  <si>
+    <t>-1.0%</t>
+  </si>
+  <si>
+    <t>-0.5%</t>
+  </si>
+  <si>
+    <t>+0.0%</t>
+  </si>
+  <si>
+    <t>+0.5%</t>
+  </si>
+  <si>
+    <t>+1.0%</t>
+  </si>
+  <si>
+    <t>+1.5%</t>
+  </si>
+  <si>
+    <t>+2.0%</t>
   </si>
   <si>
     <t>1Y</t>
@@ -192,7 +198,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.0%</c:v>
+                  <c:v>-2.0%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -227,16 +233,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>-0</c:v>
+                  <c:v>1.6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-0</c:v>
+                  <c:v>3.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-0</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -251,7 +257,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.5%</c:v>
+                  <c:v>-1.5%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -286,16 +292,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>-0.5</c:v>
+                  <c:v>1.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-1</c:v>
+                  <c:v>2.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-2.5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-5</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -310,7 +316,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>1.0%</c:v>
+                  <c:v>-1.0%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -345,16 +351,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>-1</c:v>
+                  <c:v>0.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-2</c:v>
+                  <c:v>1.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-5</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-10</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -369,7 +375,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>1.5%</c:v>
+                  <c:v>-0.5%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -404,16 +410,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>-1.5</c:v>
+                  <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-3</c:v>
+                  <c:v>0.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-7.5</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-15</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -428,7 +434,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>2.0%</c:v>
+                  <c:v>+0.0%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -463,16 +469,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>-2</c:v>
+                  <c:v>-0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-4</c:v>
+                  <c:v>-0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-10</c:v>
+                  <c:v>-0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-20</c:v>
+                  <c:v>-0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -487,7 +493,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>2.5%</c:v>
+                  <c:v>+0.5%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -522,16 +528,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>-2.5</c:v>
+                  <c:v>-0.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-5</c:v>
+                  <c:v>-0.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-12.5</c:v>
+                  <c:v>-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-25</c:v>
+                  <c:v>-4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -546,7 +552,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>3.0%</c:v>
+                  <c:v>+1.0%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -581,16 +587,134 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>-3</c:v>
+                  <c:v>-0.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>-1.6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="7"/>
+          <c:order val="7"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Liquidity Stress'!$I$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>+1.5%</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Liquidity Stress'!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1Y</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2Y</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5Y</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10Y</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Liquidity Stress'!$I$2:$I$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>-1.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-2.4</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>-6</c:v>
                 </c:pt>
+                <c:pt idx="3">
+                  <c:v>-12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="8"/>
+          <c:order val="8"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Liquidity Stress'!$J$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>+2.0%</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Liquidity Stress'!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1Y</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2Y</c:v>
+                </c:pt>
                 <c:pt idx="2">
-                  <c:v>-15</c:v>
+                  <c:v>5Y</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-30</c:v>
+                  <c:v>10Y</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Liquidity Stress'!$J$2:$J$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>-1.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-3.2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-16</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -701,15 +825,17 @@
     </c:title>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
             <c:v>Defaults per Round</c:v>
           </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
           <c:cat>
             <c:numRef>
               <c:f>'Contagion Simulation'!$A$2</c:f>
@@ -735,9 +861,10 @@
             </c:numRef>
           </c:val>
         </c:ser>
+        <c:marker val="1"/>
         <c:axId val="50020001"/>
         <c:axId val="50020002"/>
-      </c:barChart>
+      </c:lineChart>
       <c:catAx>
         <c:axId val="50020001"/>
         <c:scaling>
@@ -780,7 +907,7 @@
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="-5400000" vert="horz"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -1171,10 +1298,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:10">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1196,109 +1323,139 @@
       <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2">
+        <v>1.6</v>
+      </c>
+      <c r="C2">
+        <v>1.2</v>
+      </c>
+      <c r="D2">
+        <v>0.8</v>
+      </c>
+      <c r="E2">
+        <v>0.4</v>
+      </c>
+      <c r="F2">
         <v>-0</v>
       </c>
-      <c r="C2">
-        <v>-0.5</v>
-      </c>
-      <c r="D2">
-        <v>-1</v>
-      </c>
-      <c r="E2">
-        <v>-1.5</v>
-      </c>
-      <c r="F2">
+      <c r="G2">
+        <v>-0.4</v>
+      </c>
+      <c r="H2">
+        <v>-0.8</v>
+      </c>
+      <c r="I2">
+        <v>-1.2</v>
+      </c>
+      <c r="J2">
+        <v>-1.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3.2</v>
+      </c>
+      <c r="C3">
+        <v>2.4</v>
+      </c>
+      <c r="D3">
+        <v>1.6</v>
+      </c>
+      <c r="E3">
+        <v>0.8</v>
+      </c>
+      <c r="F3">
+        <v>-0</v>
+      </c>
+      <c r="G3">
+        <v>-0.8</v>
+      </c>
+      <c r="H3">
+        <v>-1.6</v>
+      </c>
+      <c r="I3">
+        <v>-2.4</v>
+      </c>
+      <c r="J3">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <v>6</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>-0</v>
+      </c>
+      <c r="G4">
         <v>-2</v>
       </c>
-      <c r="G2">
-        <v>-2.5</v>
-      </c>
-      <c r="H2">
-        <v>-3</v>
+      <c r="H4">
+        <v>-4</v>
+      </c>
+      <c r="I4">
+        <v>-6</v>
+      </c>
+      <c r="J4">
+        <v>-8</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="1" t="s">
+    <row r="5" spans="1:10">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>12</v>
+      </c>
+      <c r="D5">
         <v>8</v>
       </c>
-      <c r="B3">
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
         <v>-0</v>
       </c>
-      <c r="C3">
-        <v>-1</v>
-      </c>
-      <c r="D3">
-        <v>-2</v>
-      </c>
-      <c r="E3">
-        <v>-3</v>
-      </c>
-      <c r="F3">
+      <c r="G5">
         <v>-4</v>
       </c>
-      <c r="G3">
-        <v>-5</v>
-      </c>
-      <c r="H3">
-        <v>-6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
-        <v>-0</v>
-      </c>
-      <c r="C4">
-        <v>-2.5</v>
-      </c>
-      <c r="D4">
-        <v>-5</v>
-      </c>
-      <c r="E4">
-        <v>-7.5</v>
-      </c>
-      <c r="F4">
-        <v>-10</v>
-      </c>
-      <c r="G4">
-        <v>-12.5</v>
-      </c>
-      <c r="H4">
-        <v>-15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
-        <v>-0</v>
-      </c>
-      <c r="C5">
-        <v>-5</v>
-      </c>
-      <c r="D5">
-        <v>-10</v>
-      </c>
-      <c r="E5">
-        <v>-15</v>
-      </c>
-      <c r="F5">
-        <v>-20</v>
-      </c>
-      <c r="G5">
-        <v>-25</v>
-      </c>
       <c r="H5">
-        <v>-30</v>
+        <v>-8</v>
+      </c>
+      <c r="I5">
+        <v>-12</v>
+      </c>
+      <c r="J5">
+        <v>-16</v>
       </c>
     </row>
   </sheetData>
@@ -1314,30 +1471,30 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1363,7 +1520,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3">
         <v>0.8661761457749352</v>
@@ -1389,7 +1546,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B4">
         <v>0.1818249672071006</v>
@@ -1415,7 +1572,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>0.1394938606520418</v>
@@ -1441,7 +1598,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6">
         <v>0.5924145688620425</v>
@@ -1467,7 +1624,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B7">
         <v>0.8083973481164611</v>
@@ -1493,7 +1650,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B8">
         <v>0.0343885211152184</v>
@@ -1529,13 +1686,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1543,10 +1700,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance Banking Stress Testing contagion model and Excel dashboard visuals
</commit_message>
<xml_diff>
--- a/Banking_Stress_Testing_2024.xlsx
+++ b/Banking_Stress_Testing_2024.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t>-2.0%</t>
   </si>
@@ -87,7 +87,22 @@
     <t>New Defaults</t>
   </si>
   <si>
+    <t>Triggered Banks</t>
+  </si>
+  <si>
     <t>['SVB']</t>
+  </si>
+  <si>
+    <t>['SVB', 'Credit Suisse', 'JPM', 'BNP']</t>
+  </si>
+  <si>
+    <t>['UBS', 'JPM', 'BNP', 'Deutsche', 'SVB', 'Credit Suisse', 'HSBC']</t>
+  </si>
+  <si>
+    <t>['Credit Suisse', 'JPM', 'BNP']</t>
+  </si>
+  <si>
+    <t>['Deutsche', 'UBS', 'HSBC']</t>
   </si>
   <si>
     <t>[]</t>
@@ -831,31 +846,43 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Defaults per Round</c:v>
+            <c:v>Cumulative Defaults</c:v>
           </c:tx>
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Contagion Simulation'!$A$2</c:f>
+              <c:f>'Contagion Simulation'!$A$2:$A$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Contagion Simulation'!$B$2</c:f>
+              <c:f>'Contagion Simulation'!$D$2:$D$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1500,22 +1527,22 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>0.9507143064099162</v>
+        <v>0.9655000144869412</v>
       </c>
       <c r="D2">
-        <v>0.7319939418114051</v>
+        <v>0.8123957592679836</v>
       </c>
       <c r="E2">
-        <v>0.5986584841970366</v>
+        <v>0.7190609389379256</v>
       </c>
       <c r="F2">
-        <v>0.1560186404424365</v>
+        <v>0.4092130483097056</v>
       </c>
       <c r="G2">
-        <v>0.1559945203362026</v>
+        <v>0.4091961642353418</v>
       </c>
       <c r="H2">
-        <v>0.05808361216819946</v>
+        <v>0.3406585285177396</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1523,25 +1550,25 @@
         <v>14</v>
       </c>
       <c r="B3">
-        <v>0.8661761457749352</v>
+        <v>0.9063233020424546</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>0.7080725777960455</v>
+        <v>0.7956508044572318</v>
       </c>
       <c r="E3">
-        <v>0.02058449429580245</v>
+        <v>0.3144091460070617</v>
       </c>
       <c r="F3">
-        <v>0.9699098521619943</v>
+        <v>0.978936896513396</v>
       </c>
       <c r="G3">
-        <v>0.8324426408004217</v>
+        <v>0.8827098485602952</v>
       </c>
       <c r="H3">
-        <v>0.2123391106782762</v>
+        <v>0.4486373774747933</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1549,25 +1576,25 @@
         <v>15</v>
       </c>
       <c r="B4">
-        <v>0.1818249672071006</v>
+        <v>0.4272774770449704</v>
       </c>
       <c r="C4">
-        <v>0.1834045098534338</v>
+        <v>0.4283831568974036</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0.5247564316322378</v>
+        <v>0.6673295021425665</v>
       </c>
       <c r="F4">
-        <v>0.4319450186421158</v>
+        <v>0.602361513049481</v>
       </c>
       <c r="G4">
-        <v>0.2912291401980419</v>
+        <v>0.5038603981386293</v>
       </c>
       <c r="H4">
-        <v>0.6118528947223795</v>
+        <v>0.7282970263056656</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1575,25 +1602,25 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <v>0.1394938606520418</v>
+        <v>0.3976457024564293</v>
       </c>
       <c r="C5">
-        <v>0.2921446485352182</v>
+        <v>0.5045012539746527</v>
       </c>
       <c r="D5">
-        <v>0.3663618432936917</v>
+        <v>0.5564532903055842</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0.7851759613930136</v>
+        <v>0.8496231729751095</v>
       </c>
       <c r="G5">
-        <v>0.1996737821583597</v>
+        <v>0.4397716475108518</v>
       </c>
       <c r="H5">
-        <v>0.5142344384136116</v>
+        <v>0.6599641068895281</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1601,25 +1628,25 @@
         <v>17</v>
       </c>
       <c r="B6">
-        <v>0.5924145688620425</v>
+        <v>0.7146901982034297</v>
       </c>
       <c r="C6">
-        <v>0.04645041271999772</v>
+        <v>0.3325152889039984</v>
       </c>
       <c r="D6">
-        <v>0.6075448519014384</v>
+        <v>0.7252813963310069</v>
       </c>
       <c r="E6">
-        <v>0.1705241236872915</v>
+        <v>0.419366886581104</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>0.9488855372533332</v>
+        <v>0.9642198760773332</v>
       </c>
       <c r="H6">
-        <v>0.9656320330745594</v>
+        <v>0.9759424231521915</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1627,25 +1654,25 @@
         <v>18</v>
       </c>
       <c r="B7">
-        <v>0.8083973481164611</v>
+        <v>0.8658781436815227</v>
       </c>
       <c r="C7">
-        <v>0.3046137691733707</v>
+        <v>0.5132296384213595</v>
       </c>
       <c r="D7">
-        <v>0.09767211400638387</v>
+        <v>0.3683704798044687</v>
       </c>
       <c r="E7">
-        <v>0.6842330265121569</v>
+        <v>0.7789631185585097</v>
       </c>
       <c r="F7">
-        <v>0.4401524937396013</v>
+        <v>0.6081067456177209</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7">
-        <v>0.4951769101112702</v>
+        <v>0.6466238370778891</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1653,22 +1680,22 @@
         <v>19</v>
       </c>
       <c r="B8">
-        <v>0.0343885211152184</v>
+        <v>0.3240719647806529</v>
       </c>
       <c r="C8">
-        <v>0.9093204020787821</v>
+        <v>0.9365242814551474</v>
       </c>
       <c r="D8">
-        <v>0.2587799816000169</v>
+        <v>0.4811459871200118</v>
       </c>
       <c r="E8">
-        <v>0.662522284353982</v>
+        <v>0.7637655990477873</v>
       </c>
       <c r="F8">
-        <v>0.311711076089411</v>
+        <v>0.5181977532625877</v>
       </c>
       <c r="G8">
-        <v>0.5200680211778108</v>
+        <v>0.6640476148244675</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -1681,10 +1708,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -1694,16 +1721,50 @@
       <c r="C1" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>27</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tune contagion to show propagation, fix Excel chart to use Cumulative Defaults
</commit_message>
<xml_diff>
--- a/Banking_Stress_Testing_2024.xlsx
+++ b/Banking_Stress_Testing_2024.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <t>-2.0%</t>
   </si>
@@ -81,31 +81,10 @@
     <t>Round</t>
   </si>
   <si>
-    <t>Defaults</t>
-  </si>
-  <si>
     <t>New Defaults</t>
   </si>
   <si>
-    <t>Triggered Banks</t>
-  </si>
-  <si>
-    <t>['SVB']</t>
-  </si>
-  <si>
-    <t>['SVB', 'Credit Suisse', 'JPM', 'BNP']</t>
-  </si>
-  <si>
-    <t>['UBS', 'JPM', 'BNP', 'Deutsche', 'SVB', 'Credit Suisse', 'HSBC']</t>
-  </si>
-  <si>
-    <t>['Credit Suisse', 'JPM', 'BNP']</t>
-  </si>
-  <si>
-    <t>['Deutsche', 'UBS', 'HSBC']</t>
-  </si>
-  <si>
-    <t>[]</t>
+    <t>Cumulative Defaults</t>
   </si>
 </sst>
 </file>
@@ -848,41 +827,26 @@
           <c:tx>
             <c:v>Cumulative Defaults</c:v>
           </c:tx>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Contagion Simulation'!$A$2:$A$4</c:f>
+              <c:f>'Contagion Simulation'!$A$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Contagion Simulation'!$D$2:$D$4</c:f>
+              <c:f>'Contagion Simulation'!$C$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>7</c:v>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1527,22 +1491,22 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>0.9655000144869412</v>
+        <v>0.2015171140968154</v>
       </c>
       <c r="D2">
-        <v>0.8123957592679836</v>
+        <v>0.3472299500874105</v>
       </c>
       <c r="E2">
-        <v>0.7190609389379256</v>
+        <v>0.3276977356218537</v>
       </c>
       <c r="F2">
-        <v>0.4092130483097056</v>
+        <v>0.2024851416253264</v>
       </c>
       <c r="G2">
-        <v>0.4091961642353418</v>
+        <v>0.19915236922909</v>
       </c>
       <c r="H2">
-        <v>0.3406585285177396</v>
+        <v>0.3119542018978421</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1550,25 +1514,25 @@
         <v>14</v>
       </c>
       <c r="B3">
-        <v>0.9063233020424546</v>
+        <v>0.3515084983910086</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>0.7956508044572318</v>
+        <v>0.3294494716354866</v>
       </c>
       <c r="E3">
-        <v>0.3144091460070617</v>
+        <v>0.121372929912071</v>
       </c>
       <c r="F3">
-        <v>0.978936896513396</v>
+        <v>0.1803461968899578</v>
       </c>
       <c r="G3">
-        <v>0.8827098485602952</v>
+        <v>0.2526789777827141</v>
       </c>
       <c r="H3">
-        <v>0.4486373774747933</v>
+        <v>0.05441336795621621</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1576,25 +1540,25 @@
         <v>15</v>
       </c>
       <c r="B4">
-        <v>0.4272774770449704</v>
+        <v>0.1010946905290184</v>
       </c>
       <c r="C4">
-        <v>0.4283831568974036</v>
+        <v>0.1630183379481444</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0.6673295021425665</v>
+        <v>0.1790563183236937</v>
       </c>
       <c r="F4">
-        <v>0.602361513049481</v>
+        <v>0.1445652783407431</v>
       </c>
       <c r="G4">
-        <v>0.5038603981386293</v>
+        <v>0.1104968301443956</v>
       </c>
       <c r="H4">
-        <v>0.7282970263056656</v>
+        <v>0.2947343272433132</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1602,25 +1566,25 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <v>0.3976457024564293</v>
+        <v>0.2139256176738007</v>
       </c>
       <c r="C5">
-        <v>0.5045012539746527</v>
+        <v>0.2233568159407045</v>
       </c>
       <c r="D5">
-        <v>0.5564532903055842</v>
+        <v>0.1231950508574958</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0.8496231729751095</v>
+        <v>0.2406165268620911</v>
       </c>
       <c r="G5">
-        <v>0.4397716475108518</v>
+        <v>0.1259193844236645</v>
       </c>
       <c r="H5">
-        <v>0.6599641068895281</v>
+        <v>0.1709034863175575</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1628,25 +1592,25 @@
         <v>17</v>
       </c>
       <c r="B6">
-        <v>0.7146901982034297</v>
+        <v>0.1773627692521712</v>
       </c>
       <c r="C6">
-        <v>0.3325152889039984</v>
+        <v>0.1866358863576689</v>
       </c>
       <c r="D6">
-        <v>0.7252813963310069</v>
+        <v>0.1859150159252627</v>
       </c>
       <c r="E6">
-        <v>0.419366886581104</v>
+        <v>0.3863392269503714</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>0.9642198760773332</v>
+        <v>0.1319315490472855</v>
       </c>
       <c r="H6">
-        <v>0.9759424231521915</v>
+        <v>0.2136891601754855</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1654,25 +1618,25 @@
         <v>18</v>
       </c>
       <c r="B7">
-        <v>0.8658781436815227</v>
+        <v>0.1300728527031288</v>
       </c>
       <c r="C7">
-        <v>0.5132296384213595</v>
+        <v>0.2397120135642348</v>
       </c>
       <c r="D7">
-        <v>0.3683704798044687</v>
+        <v>0.09428366113132033</v>
       </c>
       <c r="E7">
-        <v>0.7789631185585097</v>
+        <v>0.07876617812509668</v>
       </c>
       <c r="F7">
-        <v>0.6081067456177209</v>
+        <v>0.2511810049407988</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7">
-        <v>0.6466238370778891</v>
+        <v>0.1543054564095856</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1680,22 +1644,22 @@
         <v>19</v>
       </c>
       <c r="B8">
-        <v>0.3240719647806529</v>
+        <v>0.2260355714508724</v>
       </c>
       <c r="C8">
-        <v>0.9365242814551474</v>
+        <v>0.185759832092432</v>
       </c>
       <c r="D8">
-        <v>0.4811459871200118</v>
+        <v>0.119926850363024</v>
       </c>
       <c r="E8">
-        <v>0.7637655990477873</v>
+        <v>0.1067676110669135</v>
       </c>
       <c r="F8">
-        <v>0.5181977532625877</v>
+        <v>0.1808058513410825</v>
       </c>
       <c r="G8">
-        <v>0.6640476148244675</v>
+        <v>0.3798208893728503</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -1708,10 +1672,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -1721,50 +1685,16 @@
       <c r="C1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3">
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
         <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>